<commit_message>
feat(controls): add control 4.15 Copilot Cowork Governance (Pillar 4)
Author net-new governance control 4.15 covering Microsoft 365 Copilot
Cowork (Frontier preview), with 4 implementation playbooks. Thread the
control-count invariant 62->63 and Pillar-4 count 14->15 through the
manifest pipeline, count gates, SPA runtime strings, vitest/pytest
suites, and narrative docs. Playbook totals 264->268 (control 245->249).

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/assessment/templates/ai-administrator-checklist.xlsx
+++ b/assessment/templates/ai-administrator-checklist.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI Administrator" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'AI Administrator'!$A$4:$I$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'AI Administrator'!$A$4:$I$12</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -513,7 +513,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Role: AI Administrator  |  FSI Copilot Governance Framework v1.4  |  7 controls</t>
+          <t>Role: AI Administrator  |  FSI Copilot Governance Framework v1.4  |  8 controls</t>
         </is>
       </c>
     </row>
@@ -598,7 +598,7 @@
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>Documentation exists describing what the Semantic Index indexes across each M365 workload in the organization; SharePoint search indexing configuration has been reviewed and sites containing regulated data are documented; Semantic Index scope has been mapped against the data classification inventory from Control 1.1; Appropriate scope controls (RSS, RCD, search exclusion) are in place for sites containing sensitive or regulated content; DSPM Activity Explorer monitoring is configured to track Copilot content retrieval patterns (Recommended and Regulated levels); Formal risk assessment of Semantic Index data processing has been conducted for regulated data types (Regulated level); Semantic Index governance posture is documented in the organization's Copilot governance documentation; Information security team has reviewed and approved the Semantic Index governance posture (Regulated level); Semantic Index data flow and architecture are documented in the organization's technology risk assessment (Regulated level); Periodic review cadence for Semantic Index governance is established (quarterly minimum)</t>
+          <t>Documented semantic-index scope policy with inclusion/exclusion criteria; List of sites excluded from indexing with business justification; Review cadence evidence (meeting minutes, policy revision date); Data classification alignment documentation</t>
         </is>
       </c>
       <c r="H5" s="5" t="inlineStr"/>
@@ -637,7 +637,7 @@
       </c>
       <c r="G6" s="7" t="inlineStr">
         <is>
-          <t>Microsoft is registered in the institution's third-party vendor inventory as an AI service provider with appropriate criticality classification; Microsoft's Copilot data handling documentation has been reviewed and key commitments documented (no training on customer data, data residency, retention); Microsoft's SOC 2 Type II report and ISO 27001 certification have been reviewed within the past 12 months; Formal vendor risk assessment has been completed using the institution's third-party risk framework (Recommended and Regulated levels); Microsoft's subprocessor list has been reviewed and AI subprocessors identified (Recommended and Regulated levels); Microsoft's DPA and Product Terms have been reviewed for AI-specific provisions (Recommended and Regulated levels); Legal counsel has reviewed contractual terms for AI service provisions (Regulated level); Fourth-party risk assessment has been conducted for AI subprocessors (Regulated level); Residual risk has been documented and risk acceptance obtained from appropriate authority; Vendor risk documentation is maintained in the regulatory examination file and includes ongoing monitoring plan (Regulated level)</t>
+          <t>Vendor risk assessment report for Microsoft Copilot (dated); Sub-processor risk evaluation covering Azure OpenAI data processing; Third-party plug-in/connector risk inventory and assessment; Annual refresh schedule or material-change trigger documentation</t>
         </is>
       </c>
       <c r="H6" s="7" t="inlineStr"/>
@@ -676,7 +676,7 @@
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>Inventory of all active Graph connectors has been completed with data source, sensitivity classification, and permission model documented; Plugin availability settings have been reviewed and non-assessed plugins disabled; SharePoint declarative agent configuration has been reviewed and agents disabled on sites containing sensitive data (unless specifically approved); Plugin approval process has been established with risk classification criteria (Recommended and Regulated levels); Security review has been conducted for all active Graph connectors (Recommended and Regulated levels); Data flow assessment has been completed for each active connector and plugin, documenting what data enters and leaves M365 (Recommended and Regulated levels); Compliance sign-off has been obtained for plugins with write access to external systems (Regulated level); Third-party extension providers are included in the vendor risk inventory (Regulated level); Extensibility change management process is documented and being followed; Extensibility governance documentation is maintained and accessible for regulatory examination (Regulated level)</t>
+          <t>Extensibility governance framework document; Approval workflow documentation for agents, plug-ins, connectors; Current extensibility inventory (agents, plug-ins, connectors, MCP); Risk classification scheme for extensibility surfaces</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr"/>
@@ -715,7 +715,7 @@
       </c>
       <c r="G8" s="7" t="inlineStr">
         <is>
-          <t>Review Copilot Tuning tenant settings — Tuning is disabled or restricted to approved groups per policy; Verify tuning access group membership — Only approved users are in the tuning-enabled Entra ID group; Review tuning request and approval workflow — Documented approval process exists with business justification requirements; Confirm data source restrictions are documented — Approved and restricted SharePoint sites for tuning are identified; Review active tuned agents inventory — List of active tuned agents with data sources and owners is current; Verify audit trail for tuning events — Tuning requests, approvals, and agent lifecycle events are logged; Confirm output supervision process (Regulated) — Periodic output review evidence exists for active tuned agents; Review open-source model control settings — External base model usage is configured per organizational policy</t>
+          <t>Model-governance review documentation for Copilot Tuning; Evaluation harness results (accuracy, bias, safety); Tuning artifact retention policy and location; Approval workflow for publishing tuned models</t>
         </is>
       </c>
       <c r="H8" s="7" t="inlineStr"/>
@@ -754,7 +754,7 @@
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>Verify FFIEC mapping documentation exists — Mapping covers all applicable FFIEC booklet requirements for Copilot; Verify Copilot is included in FFIEC CAT self-assessment — All five CAT domains reflect Copilot deployment; Verify IT risk assessment includes Copilot — Risk assessment documents Copilot as an AI technology risk; Review examiner-ready documentation packages — Packages organized by FFIEC booklet with current evidence; Verify annual FFIEC alignment review is completed — Review documentation shows mapping updates and gap remediation; Test examination response readiness — Copilot governance documentation producible within 2 business days of examiner request; Verify independent FFIEC readiness assessment — Assessment completed with findings and remediation plan; Review mock examination results — Mock examination completed with documented outcomes and improvements; Verify CAT maturity advancement plan — Plan documents target maturity levels and timeline for advancement; Verify multi-charter coordination — Documentation serves all applicable examination audiences consistently</t>
+          <t>FFIEC IT Handbook alignment assessment for Copilot; Gap analysis document with remediation plan; Coverage of Information Security, Outsourcing, and Architecture sections; Review date and next scheduled review</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr"/>
@@ -793,7 +793,7 @@
       </c>
       <c r="G10" s="7" t="inlineStr">
         <is>
-          <t>Access Copilot Dashboard in Viva Insights — Dashboard accessible to approved analysts; Review Adoption and Impact views — Current data is available in both views; Verify access restrictions — Only designated personnel can access the dashboard; Review latest leadership summary — Impact reporting exists and includes caveats; Confirm privacy posture — Aggregation and access decisions are documented; Confirm linkage to governance review — Impact data is discussed with usage and cost reporting</t>
+          <t>Viva Insights Copilot impact report with caveats applied; Review cadence documentation and most recent review date; Statistical-limitation disclaimers in leadership reports</t>
         </is>
       </c>
       <c r="H10" s="7" t="inlineStr"/>
@@ -832,20 +832,59 @@
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>Review consolidated inventory — Plugins, connectors, and governed agents are documented; Verify ownership — All published or broadly shared agents have owners; Review Agent Overview — Metrics and governance action cards are monitored; Confirm settings baseline — Allowed types, sharing, templates, and user access match policy; Review third-party or partner components — Reassessment evidence exists for higher-risk components; Confirm stale component handling — Blocked or retired items are documented</t>
+          <t>Agent and plug-in inventory with operational status; Approval workflow for new extensibility surface publication; Operational monitoring dashboard for agent health and usage; Error rate tracking and alerting configuration</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr"/>
       <c r="I11" s="5" t="inlineStr"/>
     </row>
+    <row r="12" ht="42" customHeight="1">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>4.15</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Copilot Cowork Governance</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>P4 – Operations &amp; Lifecycle</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>Baseline / Recommended / Regulated</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>Copilot admin center; Teams/Viva; Sentinel</t>
+        </is>
+      </c>
+      <c r="F12" s="7" t="inlineStr">
+        <is>
+          <t>Is Microsoft 365 Copilot Cowork (Frontier preview) governed with deliberate availability, plugin, and supervision decisions before broad enablement?</t>
+        </is>
+      </c>
+      <c r="G12" s="7" t="inlineStr">
+        <is>
+          <t>Frontier preview enrollment record for tenant and admin accounts; Cowork availability configuration (scoped group or blocked) with approval; Approved Cowork plugin inventory and connector authentication records; Deployment/pinning approvals and supervision/audit coverage evidence</t>
+        </is>
+      </c>
+      <c r="H12" s="7" t="inlineStr"/>
+      <c r="I12" s="7" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:I11"/>
+  <autoFilter ref="A4:I12"/>
   <mergeCells count="2">
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A2:I2"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="H5:H11" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Select Yes, Partial, or No" promptTitle="Status" prompt="Select response" type="list">
+    <dataValidation sqref="H5:H12" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Select Yes, Partial, or No" promptTitle="Status" prompt="Select response" type="list">
       <formula1>"Yes,Partial,No"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Regenerate assets for Cowork/Scout v1.8.0
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>

Copilot-Session: d6ed2a9a-75d8-4330-bfd0-804c1778bf8b
</commit_message>
<xml_diff>
--- a/assessment/templates/ai-administrator-checklist.xlsx
+++ b/assessment/templates/ai-administrator-checklist.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI Administrator" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'AI Administrator'!$A$4:$I$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'AI Administrator'!$A$4:$I$13</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -513,7 +513,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Role: AI Administrator  |  FSI Copilot Governance Framework v1.4  |  8 controls</t>
+          <t>Role: AI Administrator  |  FSI Copilot Governance Framework v1.8  |  9 controls</t>
         </is>
       </c>
     </row>
@@ -866,7 +866,7 @@
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
-          <t>Is Microsoft 365 Copilot Cowork (Frontier preview) governed with deliberate availability, plugin, and supervision decisions before broad enablement?</t>
+          <t>Is Microsoft 365 Copilot Cowork governed at GA with deliberate billing/discovery, model/browser, plugin/skill, and supervision decisions before broad enablement?</t>
         </is>
       </c>
       <c r="G12" s="7" t="inlineStr">
@@ -877,14 +877,53 @@
       <c r="H12" s="7" t="inlineStr"/>
       <c r="I12" s="7" t="inlineStr"/>
     </row>
+    <row r="13" ht="42" customHeight="1">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>4.16</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Microsoft Scout Governance</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>P4 – Operations &amp; Lifecycle</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Baseline / Recommended / Regulated</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>Copilot admin center; Teams/Viva; Sentinel</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>Is Microsoft Scout governed across Frontier scope, endpoint policy plus attestation, and GitHub Copilot entitlement with documented supervision and boundary risk controls before enablement?</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>Frontier enrollment and scoping record for tenant and pilot groups; Intune policy export showing Scout enablement profile assignment and effective state; Admin attestation record naming approver and completion date; GitHub Copilot Business/Enterprise entitlement export matched to pilot users; Documented default permission posture for local files, shell commands, and browser actions; Autonomous-mode and unattended-automation decision records with scope constraints; Approved MCP inventory including authentication, egress, and data-path classification; Boundary map showing M365-protected data vs GitHub/local/third-party processing surfaces; Known unsupported evidence register (local automation artifacts, local MCP output, third-party inference telemetry)</t>
+        </is>
+      </c>
+      <c r="H13" s="5" t="inlineStr"/>
+      <c r="I13" s="5" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:I12"/>
+  <autoFilter ref="A4:I13"/>
   <mergeCells count="2">
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A2:I2"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="H5:H12" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Select Yes, Partial, or No" promptTitle="Status" prompt="Select response" type="list">
+    <dataValidation sqref="H5:H13" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Select Yes, Partial, or No" promptTitle="Status" prompt="Select response" type="list">
       <formula1>"Yes,Partial,No"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
fix: [OCEAN-255] correct control 3.11 SEC citation
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/assessment/templates/ai-administrator-checklist.xlsx
+++ b/assessment/templates/ai-administrator-checklist.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI Administrator" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'AI Administrator'!$A$4:$I$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'AI Administrator'!$A$4:$I$14</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:I14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -513,7 +513,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Role: AI Administrator  |  FSI Copilot Governance Framework v1.8.0  |  9 controls</t>
+          <t>Role: AI Administrator  |  FSI Copilot Governance Framework v1.8.0  |  10 controls</t>
         </is>
       </c>
     </row>
@@ -724,12 +724,12 @@
     <row r="9" ht="42" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>3.13</t>
+          <t>3.8a</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>FFIEC IT Examination Handbook Alignment</t>
+          <t>Generative AI Model Governance for Microsoft 365 Copilot</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
@@ -749,12 +749,12 @@
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>Has FFIEC IT Handbook alignment (Information Security, Outsourcing, Architecture) been reviewed for Copilot deployment?</t>
+          <t>Has a generative-AI model-governance review (NIST AI RMF 1.0 / ISO/IEC 42001, addressing the SR 26-2 / OCC 2026-13 generative-AI exclusion) been completed for Copilot?</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>FFIEC IT Handbook alignment assessment for Copilot; Gap analysis document with remediation plan; Coverage of Information Security, Outsourcing, and Architecture sections; Review date and next scheduled review</t>
+          <t>Generative-AI governance review document for Copilot; NIST AI RMF 1.0 alignment documentation; Bias testing and safety evaluation results; Responsible-AI principles adoption evidence</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr"/>
@@ -763,17 +763,17 @@
     <row r="10" ht="42" customHeight="1">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>4.6</t>
+          <t>3.13</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>Microsoft Viva Insights and Copilot Analytics Impact Measurement</t>
+          <t>FFIEC IT Examination Handbook Alignment</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>P4 – Operations &amp; Lifecycle</t>
+          <t>P3 – Compliance &amp; Records</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
@@ -783,17 +783,17 @@
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>Copilot admin center; Teams/Viva; Sentinel</t>
+          <t>Purview audit/eDiscovery/retention; FINRA/SEC records</t>
         </is>
       </c>
       <c r="F10" s="7" t="inlineStr">
         <is>
-          <t>Are Viva Insights Copilot impact reports reviewed on a documented cadence with caveats applied?</t>
+          <t>Has FFIEC IT Handbook alignment (Information Security, Outsourcing, Architecture) been reviewed for Copilot deployment?</t>
         </is>
       </c>
       <c r="G10" s="7" t="inlineStr">
         <is>
-          <t>Viva Insights Copilot impact report with caveats applied; Review cadence documentation and most recent review date; Statistical-limitation disclaimers in leadership reports</t>
+          <t>FFIEC IT Handbook alignment assessment for Copilot; Gap analysis document with remediation plan; Coverage of Information Security, Outsourcing, and Architecture sections; Review date and next scheduled review</t>
         </is>
       </c>
       <c r="H10" s="7" t="inlineStr"/>
@@ -802,12 +802,12 @@
     <row r="11" ht="42" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>4.13</t>
+          <t>4.6</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Copilot Extensibility and Agent Operations Governance</t>
+          <t>Microsoft Viva Insights and Copilot Analytics Impact Measurement</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
@@ -827,12 +827,12 @@
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>Are extensibility surfaces (declarative agents, MCP, plug-ins) governed by an approval and inventory process before publication?</t>
+          <t>Are Viva Insights Copilot impact reports reviewed on a documented cadence with caveats applied?</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>Agent and plug-in inventory with operational status; Approval workflow for new extensibility surface publication; Operational monitoring dashboard for agent health and usage; Error rate tracking and alerting configuration</t>
+          <t>Viva Insights Copilot impact report with caveats applied; Review cadence documentation and most recent review date; Statistical-limitation disclaimers in leadership reports</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr"/>
@@ -841,12 +841,12 @@
     <row r="12" ht="42" customHeight="1">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>4.15</t>
+          <t>4.13</t>
         </is>
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>Copilot Cowork Governance</t>
+          <t>Copilot Extensibility and Agent Operations Governance</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
@@ -866,12 +866,12 @@
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
-          <t>Is Microsoft 365 Copilot Cowork governed at GA with deliberate billing/discovery, model/browser, plugin/skill, and supervision decisions before broad enablement?</t>
+          <t>Are extensibility surfaces (declarative agents, MCP, plug-ins) governed by an approval and inventory process before publication?</t>
         </is>
       </c>
       <c r="G12" s="7" t="inlineStr">
         <is>
-          <t>Usage-based billing scope export (user/group assignments) with approver; Discovery-setting decision record and access-request workflow evidence; Model-policy record for Anthropic family and Claude Fable 5 (Preview); Cowork Browsing tenant-toggle decision tied to browser-control review; Consumption-limit policy and recent spend/consumption report; Approved plugin, uploaded package, and custom-skill inventory with owner; Purview coverage evidence (audit/eDiscovery/DLP alignment) and gap log</t>
+          <t>Agent and plug-in inventory with operational status; Approval workflow for new extensibility surface publication; Operational monitoring dashboard for agent health and usage; Error rate tracking and alerting configuration</t>
         </is>
       </c>
       <c r="H12" s="7" t="inlineStr"/>
@@ -880,12 +880,12 @@
     <row r="13" ht="42" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>4.16</t>
+          <t>4.15</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Microsoft Scout Governance</t>
+          <t>Copilot Cowork Governance</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
@@ -905,25 +905,64 @@
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>Is Microsoft Scout governed across Frontier scope, endpoint policy plus attestation, and GitHub Copilot entitlement with documented supervision and boundary risk controls before enablement?</t>
+          <t>Is Microsoft 365 Copilot Cowork governed at GA with deliberate billing/discovery, model/browser, plugin/skill, and supervision decisions before broad enablement?</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>Frontier enrollment and scoping record for tenant and pilot groups; Intune policy export showing Scout enablement profile assignment and effective state; Admin attestation record naming approver and completion date; GitHub Copilot Business/Enterprise entitlement export matched to pilot users; Documented default permission posture for local files, shell commands, and browser actions; Autonomous-mode and unattended-automation decision records with scope constraints; Approved MCP inventory including authentication, egress, and data-path classification; Boundary map showing M365-protected data vs GitHub/local/third-party processing surfaces; Known unsupported evidence register (local automation artifacts, local MCP output, third-party inference telemetry)</t>
+          <t>Usage-based billing scope export (user/group assignments) with approver; Discovery-setting decision record and access-request workflow evidence; Model-policy record for Anthropic family and Claude Fable 5 (Preview); Cowork Browsing tenant-toggle decision tied to browser-control review; Consumption-limit policy and recent spend/consumption report; Approved plugin, uploaded package, and custom-skill inventory with owner; Purview coverage evidence (audit/eDiscovery/DLP alignment) and gap log</t>
         </is>
       </c>
       <c r="H13" s="5" t="inlineStr"/>
       <c r="I13" s="5" t="inlineStr"/>
     </row>
+    <row r="14" ht="42" customHeight="1">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>4.16</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Microsoft Scout Governance</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>P4 – Operations &amp; Lifecycle</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>Baseline / Recommended / Regulated</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>Copilot admin center; Teams/Viva; Sentinel</t>
+        </is>
+      </c>
+      <c r="F14" s="7" t="inlineStr">
+        <is>
+          <t>Is Microsoft Scout governed across Frontier scope, endpoint policy plus attestation, and GitHub Copilot entitlement with documented supervision and boundary risk controls before enablement?</t>
+        </is>
+      </c>
+      <c r="G14" s="7" t="inlineStr">
+        <is>
+          <t>Frontier enrollment and scoping record for tenant and pilot groups; Intune policy export showing Scout enablement profile assignment and effective state; Admin attestation record naming approver and completion date; GitHub Copilot Business/Enterprise entitlement export matched to pilot users; Documented default permission posture for local files, shell commands, and browser actions; Autonomous-mode and unattended-automation decision records with scope constraints; Approved MCP inventory including authentication, egress, and data-path classification; Boundary map showing M365-protected data vs GitHub/local/third-party processing surfaces; Known unsupported evidence register (local automation artifacts, local MCP output, third-party inference telemetry)</t>
+        </is>
+      </c>
+      <c r="H14" s="7" t="inlineStr"/>
+      <c r="I14" s="7" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:I13"/>
+  <autoFilter ref="A4:I14"/>
   <mergeCells count="2">
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A2:I2"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="H5:H13" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Select Yes, Partial, or No" promptTitle="Status" prompt="Select response" type="list">
+    <dataValidation sqref="H5:H14" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Select Yes, Partial, or No" promptTitle="Status" prompt="Select response" type="list">
       <formula1>"Yes,Partial,No"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>